<commit_message>
Updated all the files new version
</commit_message>
<xml_diff>
--- a/ERP Report/PICS/Sr.Super60_Nucleus(Adv)/P1/K.xlsx
+++ b/ERP Report/PICS/Sr.Super60_Nucleus(Adv)/P1/K.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SRINIVASU(BNG11531)\ECITY\SNAPSHOT 2026-2027\Sr\11)14-06-2026_Sr.Super60_NUCLEUS-BT_Jee-Adv(2023-P1)_WTA-52_Q. Paper With Key &amp; Sol's\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SRINIVASU(BNG11531)\ECITY\SNAPSHOT 2026-2027\Sr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77FDD2F-E28C-4E61-9024-ECD5D3AC55BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1AEA47-766B-4F41-B8A9-3D94E7C75232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="120" yWindow="600" windowWidth="20370" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KEY" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="12">
   <si>
     <t>Q_No</t>
   </si>
@@ -28,31 +28,34 @@
     <t>Key</t>
   </si>
   <si>
-    <t>ABC</t>
+    <t>C</t>
   </si>
   <si>
-    <t>BC</t>
+    <t>B</t>
+  </si>
+  <si>
+    <t>AB</t>
+  </si>
+  <si>
+    <t>AC</t>
   </si>
   <si>
     <t>ABCD</t>
   </si>
   <si>
-    <t>C</t>
+    <t>D</t>
   </si>
   <si>
     <t>A</t>
   </si>
   <si>
-    <t>D</t>
+    <t>BD</t>
   </si>
   <si>
-    <t>B</t>
+    <t>ABC</t>
   </si>
   <si>
-    <t>ACD</t>
-  </si>
-  <si>
-    <t>AC</t>
+    <t>BC</t>
   </si>
 </sst>
 </file>
@@ -1113,7 +1116,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1121,7 +1124,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1129,7 +1132,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.2">
@@ -1137,7 +1140,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1153,7 +1156,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2">
-        <v>402</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1161,7 +1164,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2">
-        <v>4</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1169,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2">
-        <v>72</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1177,7 +1180,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="2">
-        <v>819</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1185,7 +1188,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="2">
-        <v>108</v>
+        <v>361</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1193,7 +1196,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="2">
-        <v>32</v>
+        <v>280</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1201,7 +1204,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1209,7 +1212,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1217,7 +1220,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1225,7 +1228,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -1233,7 +1236,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -1241,7 +1244,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -1249,7 +1252,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
@@ -1257,7 +1260,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
@@ -1265,7 +1268,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
@@ -1273,7 +1276,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
@@ -1281,7 +1284,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -1289,7 +1292,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="2">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
@@ -1297,7 +1300,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="2">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
@@ -1305,7 +1308,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
@@ -1313,7 +1316,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="2">
-        <v>2</v>
+        <v>93</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
@@ -1321,7 +1324,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
@@ -1329,7 +1332,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="2">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -1337,7 +1340,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
@@ -1345,7 +1348,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
@@ -1353,7 +1356,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
@@ -1361,7 +1364,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
@@ -1369,7 +1372,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
@@ -1377,7 +1380,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
@@ -1385,7 +1388,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
@@ -1393,7 +1396,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
@@ -1401,7 +1404,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
@@ -1409,7 +1412,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
@@ -1417,7 +1420,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
@@ -1425,7 +1428,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="2">
-        <v>4</v>
+        <v>24</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
@@ -1433,7 +1436,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
@@ -1441,7 +1444,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="2">
-        <v>9</v>
+        <v>268</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
@@ -1449,7 +1452,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="2">
-        <v>98</v>
+        <v>162</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
@@ -1457,7 +1460,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="2">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
@@ -1465,7 +1468,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="2">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -1473,7 +1476,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
@@ -1489,7 +1492,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
@@ -1497,7 +1500,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>